<commit_message>
max mau -300 deff eatch part
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/37_UnitHead/UnitHead.xlsx
+++ b/gu_in/Item.edf/37_UnitHead/UnitHead.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153D6F27-3B37-4C8C-8E63-3C7EAFFC0F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E794F8B-C4A2-4A7D-A1AA-81B44F1A01A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -826,7 +826,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -842,8 +842,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -863,6 +870,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -903,11 +915,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -915,9 +928,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -6687,168 +6704,168 @@
       </c>
       <c r="BB33" s="3"/>
     </row>
-    <row r="34" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:54" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="7">
         <v>5</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="E34" s="4">
-        <v>0</v>
-      </c>
-      <c r="F34" s="4" t="s">
+      <c r="E34" s="7">
+        <v>0</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="G34" s="3">
-        <v>-1</v>
-      </c>
-      <c r="H34" s="3">
-        <v>-1</v>
-      </c>
-      <c r="I34" s="3">
-        <v>-1</v>
-      </c>
-      <c r="J34" s="3">
-        <v>0</v>
-      </c>
-      <c r="K34" s="3">
-        <v>0</v>
-      </c>
-      <c r="L34" s="4">
+      <c r="G34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="I34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="J34" s="8">
+        <v>0</v>
+      </c>
+      <c r="K34" s="8">
+        <v>0</v>
+      </c>
+      <c r="L34" s="7">
         <v>48</v>
       </c>
-      <c r="M34" s="4">
-        <v>-1</v>
-      </c>
-      <c r="N34" s="4">
-        <v>2</v>
-      </c>
-      <c r="O34" s="4">
+      <c r="M34" s="7">
+        <v>-1</v>
+      </c>
+      <c r="N34" s="7">
+        <v>2</v>
+      </c>
+      <c r="O34" s="7">
         <v>93</v>
       </c>
-      <c r="P34" s="4">
-        <v>-1</v>
-      </c>
-      <c r="Q34" s="4">
-        <v>-1</v>
-      </c>
-      <c r="R34" s="3">
+      <c r="P34" s="7">
+        <v>-1</v>
+      </c>
+      <c r="Q34" s="7">
+        <v>-1</v>
+      </c>
+      <c r="R34" s="8">
         <v>1</v>
       </c>
-      <c r="S34" s="3">
-        <v>0</v>
-      </c>
-      <c r="T34" s="3">
-        <v>0</v>
-      </c>
-      <c r="U34" s="3">
-        <v>0</v>
-      </c>
-      <c r="V34" s="3">
-        <v>0</v>
-      </c>
-      <c r="W34" s="3">
-        <v>-1</v>
-      </c>
-      <c r="X34" s="3">
-        <v>-1</v>
-      </c>
-      <c r="Y34" s="3">
+      <c r="S34" s="8">
+        <v>0</v>
+      </c>
+      <c r="T34" s="8">
+        <v>0</v>
+      </c>
+      <c r="U34" s="8">
+        <v>0</v>
+      </c>
+      <c r="V34" s="8">
+        <v>0</v>
+      </c>
+      <c r="W34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="X34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="Y34" s="8">
         <v>247</v>
       </c>
-      <c r="Z34" s="3">
-        <v>50</v>
-      </c>
-      <c r="AA34" s="3">
-        <v>50</v>
-      </c>
-      <c r="AB34" s="4">
-        <v>1325</v>
-      </c>
-      <c r="AC34" s="3">
-        <v>50</v>
-      </c>
-      <c r="AD34" s="3">
-        <v>-1</v>
-      </c>
-      <c r="AE34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI34" s="4">
-        <v>0</v>
-      </c>
-      <c r="AJ34" s="4">
+      <c r="Z34" s="8">
+        <v>50</v>
+      </c>
+      <c r="AA34" s="8">
+        <v>50</v>
+      </c>
+      <c r="AB34" s="7">
+        <v>1025</v>
+      </c>
+      <c r="AC34" s="8">
+        <v>50</v>
+      </c>
+      <c r="AD34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="AE34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AF34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AG34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AH34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AI34" s="7">
+        <v>0</v>
+      </c>
+      <c r="AJ34" s="7">
         <v>1900000</v>
       </c>
-      <c r="AK34" s="4">
+      <c r="AK34" s="7">
         <v>1</v>
       </c>
-      <c r="AL34" s="4">
+      <c r="AL34" s="7">
         <v>1</v>
       </c>
-      <c r="AM34" s="3">
+      <c r="AM34" s="8">
         <v>38000</v>
       </c>
-      <c r="AN34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AO34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AP34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AQ34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AR34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AS34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AT34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AV34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AW34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AX34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AY34" s="3" t="str">
+      <c r="AN34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AO34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AP34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AQ34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AR34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AS34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AT34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AU34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AV34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AW34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AX34" s="8">
+        <v>0</v>
+      </c>
+      <c r="AY34" s="8" t="str">
         <f t="shared" si="0"/>
         <v>tunhe032</v>
       </c>
-      <c r="AZ34" s="4">
-        <v>-1</v>
-      </c>
-      <c r="BA34" s="4">
-        <v>2</v>
-      </c>
-      <c r="BB34" s="3"/>
+      <c r="AZ34" s="7">
+        <v>-1</v>
+      </c>
+      <c r="BA34" s="7">
+        <v>2</v>
+      </c>
+      <c r="BB34" s="8"/>
     </row>
     <row r="35" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
@@ -20617,7 +20634,7 @@
       </c>
       <c r="AB34">
         <f>UnitHead!AB34</f>
-        <v>1325</v>
+        <v>1025</v>
       </c>
       <c r="AC34" s="5">
         <v>0</v>

</xml_diff>

<commit_message>
max black mau price 800M
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/37_UnitHead/UnitHead.xlsx
+++ b/gu_in/Item.edf/37_UnitHead/UnitHead.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E794F8B-C4A2-4A7D-A1AA-81B44F1A01A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C5F2F2-5DC1-48EB-B78C-88CE430AC908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6811,7 +6811,7 @@
         <v>0</v>
       </c>
       <c r="AJ34" s="7">
-        <v>1900000</v>
+        <v>90909382</v>
       </c>
       <c r="AK34" s="7">
         <v>1</v>
@@ -20572,7 +20572,7 @@
       </c>
       <c r="I34">
         <f>UnitHead!AJ34</f>
-        <v>1900000</v>
+        <v>90909382</v>
       </c>
       <c r="J34">
         <f>UnitHead!AK34</f>

</xml_diff>